<commit_message>
login system and front-end
</commit_message>
<xml_diff>
--- a/data/hotel.xlsx
+++ b/data/hotel.xlsx
@@ -5,6 +5,7 @@
     <sheet name="rooms" sheetId="1" r:id="rId1"/>
     <sheet name="room_types" sheetId="2" r:id="rId2"/>
     <sheet name="bookings" sheetId="3" r:id="rId3"/>
+    <sheet name="users" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -830,6 +831,252 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B0006</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>102</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">สมชาย ใจดี</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">081-234-5678</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">somchai@gmail.com</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-01</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-02</t>
+        </is>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1200</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wait</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-01 13:32:22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">username</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">password</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">full_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phone</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin123</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">System Administrator</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">081-000-0001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin@hotel.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">staff</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">staff123</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">staff</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Front Desk Staff</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">081-000-0002</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">staff@hotel.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guest</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guest123</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guest</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">สมชาย ใจดี</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">081-234-5678</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">somchai@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">newguest</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pass123</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guest</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test User</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">089-999-8888</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">test@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PPP</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>1234</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guest</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PPP</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>1234</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PP@gmail.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>